<commit_message>
Add Liteon forecast sheet validation
Implement Liteon-specific validation in validate_forecast_format: when username is 'liteon' read the 'Daily+Weekly+Monthly' sheet and verify presence of fixed header labels at specific cell positions, returning up to 5 missing-label messages on failure. Preserve existing template-based column-count check for other customers and simplify non-Liteon read behavior. Also update compare/liteon/transit.xlsx and remove several obsolete sample ERP/forecast XLSX files.
</commit_message>
<xml_diff>
--- a/compare/liteon/transit.xlsx
+++ b/compare/liteon/transit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\business_forecasting_pc\compare\pegatron\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\business_forecasting_lite\compare\liteon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D9FF022-19BC-40E3-962D-39A269870E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CFC0BD2-CDAA-4172-9218-016292200D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0FF2FD81-0BF5-4549-99BF-040A85CE21B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0FF2FD81-0BF5-4549-99BF-040A85CE21B2}"/>
   </bookViews>
   <sheets>
     <sheet name="在途清單" sheetId="1" r:id="rId1"/>
@@ -68,23 +68,55 @@
     <t>週別</t>
   </si>
   <si>
+    <t>Ordered Item</t>
+  </si>
+  <si>
+    <r>
+      <t>11</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">訂單&gt;送貨地點
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>32</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>訂單&gt;倉庫</t>
+    </r>
+  </si>
+  <si>
     <t>ETA</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Line 客戶採購單號</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ordered Item</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -92,13 +124,6 @@
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
@@ -110,11 +135,34 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="新細明體"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="細明體"/>
+      <family val="3"/>
       <charset val="136"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -127,13 +175,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE7F3FD"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF4C68A2"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,20 +216,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -471,47 +517,49 @@
   <dimension ref="A1:L155"/>
   <sheetFormatPr defaultColWidth="18" defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="29.21875" customWidth="1"/>
-    <col min="12" max="12" width="21.6640625" customWidth="1"/>
+    <col min="1" max="4" width="18" style="5"/>
+    <col min="5" max="5" width="23.6640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="29.21875" style="5" customWidth="1"/>
+    <col min="7" max="11" width="18" style="5"/>
+    <col min="12" max="12" width="21.6640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -670,7 +718,7 @@
     <row r="155" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="A1:L1" xr:uid="{FC45BFD8-7652-4605-B8FE-1B86FB991E70}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use dynamic columns for Liteon Transit mapping
Replace hardcoded Transit column indices and ERP-derived location->type map with dynamic column lookups for Liteon transit processing. The code now finds 訂單型態, 送貨地點 and 倉庫 columns via find_column_by_name, validates presence (returns an error JSON if missing), and determines 客戶需求地區 by reading the order-type prefix (11 -> use 送貨地點, 32 -> use 倉庫). Added informative prints and simplified fallback behavior. Also updates compare/liteon/transit.xlsx (binary) and adjusts docs/SP_...md to reflect revised module effort estimates (total hours updated from 78 to 160).
</commit_message>
<xml_diff>
--- a/compare/liteon/transit.xlsx
+++ b/compare/liteon/transit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\business_forecasting_lite\compare\liteon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CFC0BD2-CDAA-4172-9218-016292200D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F96DA04-818E-4A80-95FB-7517F778573E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0FF2FD81-0BF5-4549-99BF-040A85CE21B2}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="在途清單" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">在途清單!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">在途清單!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Tw</t>
   </si>
@@ -71,52 +71,26 @@
     <t>Ordered Item</t>
   </si>
   <si>
-    <r>
-      <t>11</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="細明體"/>
-        <family val="3"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">訂單&gt;送貨地點
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Tahoma"/>
-        <family val="2"/>
-      </rPr>
-      <t>32</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="細明體"/>
-        <family val="3"/>
-        <charset val="136"/>
-      </rPr>
-      <t>訂單&gt;倉庫</t>
-    </r>
-  </si>
-  <si>
     <t>ETA</t>
+  </si>
+  <si>
+    <t>訂單型態</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>送貨地點</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>倉庫</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -145,23 +119,15 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Tahoma"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="細明體"/>
-      <family val="3"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
+      <name val="Microsoft JhengHei"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -216,7 +182,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -225,11 +191,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -514,17 +480,17 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
-  <sheetFormatPr defaultColWidth="18" defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N155"/>
+  <sheetFormatPr defaultColWidth="18" defaultRowHeight="16.2"/>
   <cols>
-    <col min="1" max="4" width="18" style="5"/>
-    <col min="5" max="5" width="23.6640625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="29.21875" style="5" customWidth="1"/>
-    <col min="7" max="11" width="18" style="5"/>
-    <col min="12" max="12" width="21.6640625" style="5" customWidth="1"/>
+    <col min="1" max="4" width="18" style="4"/>
+    <col min="5" max="5" width="23.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="29.21875" style="4" customWidth="1"/>
+    <col min="7" max="13" width="18" style="4"/>
+    <col min="14" max="14" width="21.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="26.4" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -555,169 +521,175 @@
       <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="101" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="102" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="104" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="105" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="106" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="107" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="108" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="109" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="110" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="111" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="113" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="114" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="115" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="116" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="117" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="118" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="119" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="120" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="121" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="122" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="123" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="124" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="125" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="126" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="127" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="128" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="129" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="130" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="131" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="132" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="133" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="134" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="135" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="136" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="137" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="138" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="139" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="140" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="141" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="142" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="143" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="144" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="145" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="146" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="147" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="148" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="149" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="150" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="151" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="152" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="153" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="154" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="155" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="3" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="4" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="5" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="6" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="7" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="8" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="9" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="10" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="11" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="12" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="13" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="14" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="15" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="16" spans="1:14" ht="14.4" customHeight="1"/>
+    <row r="17" ht="14.4" customHeight="1"/>
+    <row r="18" ht="14.4" customHeight="1"/>
+    <row r="19" ht="14.4" customHeight="1"/>
+    <row r="20" ht="14.4" customHeight="1"/>
+    <row r="21" ht="14.4" customHeight="1"/>
+    <row r="22" ht="14.4" customHeight="1"/>
+    <row r="23" ht="14.4" customHeight="1"/>
+    <row r="24" ht="14.4" customHeight="1"/>
+    <row r="25" ht="14.4" customHeight="1"/>
+    <row r="26" ht="14.4" customHeight="1"/>
+    <row r="27" ht="14.4" customHeight="1"/>
+    <row r="28" ht="14.4" customHeight="1"/>
+    <row r="29" ht="14.4" customHeight="1"/>
+    <row r="30" ht="14.4" customHeight="1"/>
+    <row r="31" ht="14.4" customHeight="1"/>
+    <row r="32" ht="14.4" customHeight="1"/>
+    <row r="33" ht="14.4" customHeight="1"/>
+    <row r="34" ht="14.4" customHeight="1"/>
+    <row r="35" ht="14.4" customHeight="1"/>
+    <row r="36" ht="14.4" customHeight="1"/>
+    <row r="37" ht="14.4" customHeight="1"/>
+    <row r="38" ht="14.4" customHeight="1"/>
+    <row r="39" ht="14.4" customHeight="1"/>
+    <row r="40" ht="14.4" customHeight="1"/>
+    <row r="41" ht="14.4" customHeight="1"/>
+    <row r="42" ht="14.4" customHeight="1"/>
+    <row r="43" ht="14.4" customHeight="1"/>
+    <row r="44" ht="14.4" customHeight="1"/>
+    <row r="45" ht="14.4" customHeight="1"/>
+    <row r="46" ht="14.4" customHeight="1"/>
+    <row r="47" ht="14.4" customHeight="1"/>
+    <row r="48" ht="14.4" customHeight="1"/>
+    <row r="49" ht="14.4" customHeight="1"/>
+    <row r="50" ht="14.4" customHeight="1"/>
+    <row r="51" ht="14.4" customHeight="1"/>
+    <row r="52" ht="14.4" customHeight="1"/>
+    <row r="53" ht="14.4" customHeight="1"/>
+    <row r="54" ht="14.4" customHeight="1"/>
+    <row r="55" ht="14.4" customHeight="1"/>
+    <row r="56" ht="14.4" customHeight="1"/>
+    <row r="57" ht="14.4" customHeight="1"/>
+    <row r="58" ht="14.4" customHeight="1"/>
+    <row r="59" ht="14.4" customHeight="1"/>
+    <row r="60" ht="14.4" customHeight="1"/>
+    <row r="61" ht="14.4" customHeight="1"/>
+    <row r="62" ht="14.4" customHeight="1"/>
+    <row r="63" ht="14.4" customHeight="1"/>
+    <row r="64" ht="14.4" customHeight="1"/>
+    <row r="65" ht="14.4" customHeight="1"/>
+    <row r="66" ht="14.4" customHeight="1"/>
+    <row r="67" ht="14.4" customHeight="1"/>
+    <row r="68" ht="14.4" customHeight="1"/>
+    <row r="69" ht="14.4" customHeight="1"/>
+    <row r="70" ht="14.4" customHeight="1"/>
+    <row r="71" ht="14.4" customHeight="1"/>
+    <row r="72" ht="14.4" customHeight="1"/>
+    <row r="73" ht="14.4" customHeight="1"/>
+    <row r="74" ht="14.4" customHeight="1"/>
+    <row r="75" ht="14.4" customHeight="1"/>
+    <row r="76" ht="14.4" customHeight="1"/>
+    <row r="77" ht="14.4" customHeight="1"/>
+    <row r="78" ht="14.4" customHeight="1"/>
+    <row r="79" ht="14.4" customHeight="1"/>
+    <row r="80" ht="14.4" customHeight="1"/>
+    <row r="81" ht="14.4" customHeight="1"/>
+    <row r="82" ht="14.4" customHeight="1"/>
+    <row r="83" ht="14.4" customHeight="1"/>
+    <row r="84" ht="14.4" customHeight="1"/>
+    <row r="85" ht="14.4" customHeight="1"/>
+    <row r="86" ht="14.4" customHeight="1"/>
+    <row r="87" ht="14.4" customHeight="1"/>
+    <row r="88" ht="14.4" customHeight="1"/>
+    <row r="89" ht="14.4" customHeight="1"/>
+    <row r="90" ht="14.4" customHeight="1"/>
+    <row r="91" ht="14.4" customHeight="1"/>
+    <row r="92" ht="14.4" customHeight="1"/>
+    <row r="93" ht="14.4" customHeight="1"/>
+    <row r="94" ht="14.4" customHeight="1"/>
+    <row r="95" ht="14.4" customHeight="1"/>
+    <row r="96" ht="14.4" customHeight="1"/>
+    <row r="97" ht="14.4" customHeight="1"/>
+    <row r="98" ht="14.4" customHeight="1"/>
+    <row r="99" ht="14.4" customHeight="1"/>
+    <row r="100" ht="14.4" customHeight="1"/>
+    <row r="101" ht="14.4" customHeight="1"/>
+    <row r="102" ht="14.4" customHeight="1"/>
+    <row r="103" ht="14.4" customHeight="1"/>
+    <row r="104" ht="14.4" customHeight="1"/>
+    <row r="105" ht="14.4" customHeight="1"/>
+    <row r="106" ht="14.4" customHeight="1"/>
+    <row r="107" ht="14.4" customHeight="1"/>
+    <row r="108" ht="14.4" customHeight="1"/>
+    <row r="109" ht="14.4" customHeight="1"/>
+    <row r="110" ht="14.4" customHeight="1"/>
+    <row r="111" ht="14.4" customHeight="1"/>
+    <row r="112" ht="14.4" customHeight="1"/>
+    <row r="113" ht="14.4" customHeight="1"/>
+    <row r="114" ht="14.4" customHeight="1"/>
+    <row r="115" ht="14.4" customHeight="1"/>
+    <row r="116" ht="14.4" customHeight="1"/>
+    <row r="117" ht="14.4" customHeight="1"/>
+    <row r="118" ht="14.4" customHeight="1"/>
+    <row r="119" ht="14.4" customHeight="1"/>
+    <row r="120" ht="14.4" customHeight="1"/>
+    <row r="121" ht="14.4" customHeight="1"/>
+    <row r="122" ht="14.4" customHeight="1"/>
+    <row r="123" ht="14.4" customHeight="1"/>
+    <row r="124" ht="14.4" customHeight="1"/>
+    <row r="125" ht="14.4" customHeight="1"/>
+    <row r="126" ht="14.4" customHeight="1"/>
+    <row r="127" ht="14.4" customHeight="1"/>
+    <row r="128" ht="14.4" customHeight="1"/>
+    <row r="129" ht="14.4" customHeight="1"/>
+    <row r="130" ht="14.4" customHeight="1"/>
+    <row r="131" ht="14.4" customHeight="1"/>
+    <row r="132" ht="14.4" customHeight="1"/>
+    <row r="133" ht="14.4" customHeight="1"/>
+    <row r="134" ht="14.4" customHeight="1"/>
+    <row r="135" ht="14.4" customHeight="1"/>
+    <row r="136" ht="14.4" customHeight="1"/>
+    <row r="137" ht="14.4" customHeight="1"/>
+    <row r="138" ht="14.4" customHeight="1"/>
+    <row r="139" ht="14.4" customHeight="1"/>
+    <row r="140" ht="14.4" customHeight="1"/>
+    <row r="141" ht="14.4" customHeight="1"/>
+    <row r="142" ht="14.4" customHeight="1"/>
+    <row r="143" ht="14.4" customHeight="1"/>
+    <row r="144" ht="14.4" customHeight="1"/>
+    <row r="145" ht="14.4" customHeight="1"/>
+    <row r="146" ht="14.4" customHeight="1"/>
+    <row r="147" ht="14.4" customHeight="1"/>
+    <row r="148" ht="14.4" customHeight="1"/>
+    <row r="149" ht="14.4" customHeight="1"/>
+    <row r="150" ht="14.4" customHeight="1"/>
+    <row r="151" ht="14.4" customHeight="1"/>
+    <row r="152" ht="14.4" customHeight="1"/>
+    <row r="153" ht="14.4" customHeight="1"/>
+    <row r="154" ht="14.4" customHeight="1"/>
+    <row r="155" ht="14.4" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:L1" xr:uid="{FC45BFD8-7652-4605-B8FE-1B86FB991E70}"/>
+  <autoFilter ref="A1:N1" xr:uid="{FC45BFD8-7652-4605-B8FE-1B86FB991E70}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>